<commit_message>
Leads: 2026-10-21 13:43 UTC (cycle 4)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-21.xlsx
+++ b/output/leads_2026-10-21.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -563,6 +563,66 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>All Phase Construction</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>allphaseconstructionpa.com</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>https://allphaseconstructionpa.com/services/roofing/</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Why Homeowners</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>allphaseconstruction@frontiernet.net</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>717-371-6451</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Lancaster PA</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>96</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>roof repair company Lancaster PA</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-21 13:49 UTC (cycle 8)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-21.xlsx
+++ b/output/leads_2026-10-21.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -623,6 +623,66 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Caliber Roofing &amp; Construction LLC | Roofers in El Paso, TX</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>caliber-roofing.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://caliber-roofing.com/</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>El Paso</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>info@caliber-roofing.com</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>(915) 820-5483</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>El Paso TX</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>90</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>roofing contractor El Paso TX</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-21 20:04 UTC (cycle 4)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-21.xlsx
+++ b/output/leads_2026-10-21.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -683,6 +683,122 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Licensed HVAC Services, AC Repair, Air Conditioner Installation, HVAC System Rep</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>hamiltonheatandair.com</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://www.hamiltonheatandair.com/</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Family Business</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>info@hamiltonheatandair.com</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>918-576-6835</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Tulsa OK</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>100</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>air conditioning repair Tulsa OK</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Residential &amp; Commercial Roofing, Siding and More! | Landmark Roofing</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>landmarkroofingexperts.com</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://www.landmarkroofingexperts.com/</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>a861d7b8f749b2d845c187a0aae4c1e7@errors.reusser.io</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>260-610-7006</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Fort Wayne IN</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>90</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>residential roofing company Fort Wayne IN</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-21 20:11 UTC (cycle 9)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-21.xlsx
+++ b/output/leads_2026-10-21.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -764,7 +764,6 @@
           <t>https://www.landmarkroofingexperts.com/</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>a861d7b8f749b2d845c187a0aae4c1e7@errors.reusser.io</t>
@@ -794,6 +793,62 @@
         </is>
       </c>
       <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>El Dorado Heating and Cool LLC</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>eldoradohvac.com</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://eldoradohvac.com/</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>alex@eldoradohvac.com</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>239-404-6797</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Naples FL</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>90</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>heating and cooling company Naples FL</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
         <is>
           <t>2026-10-21</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-21 20:14 UTC (cycle 11)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-21.xlsx
+++ b/output/leads_2026-10-21.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -819,7 +819,6 @@
           <t>https://eldoradohvac.com/</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>alex@eldoradohvac.com</t>
@@ -849,6 +848,62 @@
         </is>
       </c>
       <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Roofing Contractors Kenosha, WI | Racine, WI</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>mayroofing.com</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://www.mayroofing.com/</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>mayroofing@wi.rr.com</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>(262) 843-3603</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Kenosha WI</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>96</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>roofing contractor Kenosha WI</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
         <is>
           <t>2026-10-21</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-21 20:16 UTC (cycle 12)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-21.xlsx
+++ b/output/leads_2026-10-21.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -874,7 +874,6 @@
           <t>https://www.mayroofing.com/</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>mayroofing@wi.rr.com</t>
@@ -904,6 +903,122 @@
         </is>
       </c>
       <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Plumbing Company Toledo, OH</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>rootwrestler.com</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://www.rootwrestler.com/</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>rootwrestler@gmail.com</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>(419) 330-8225</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Toledo OH</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>100</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>plumbing company Toledo OH</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Roof Repair in Minneapolis, MN | Same-Day Local Service</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>roofingprosminneapolismn.com</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://roofingprosminneapolismn.com/</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Roof Repair</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>info@roofingprosminneapolismn.com</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>(612) 509-5425</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Minneapolis MN</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>90</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>roof repair company Minneapolis MN</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
         <is>
           <t>2026-10-21</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-21 20:17 UTC (cycle 13)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-21.xlsx
+++ b/output/leads_2026-10-21.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -929,7 +929,6 @@
           <t>https://www.rootwrestler.com/</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>rootwrestler@gmail.com</t>
@@ -1019,6 +1018,62 @@
         </is>
       </c>
       <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>A Honorable Roofing</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>albuquerqueroofingpro.com</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://albuquerqueroofingpro.com/services/metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>ahroofingco28@gmail.com</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>505-864-6790</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Albuquerque NM</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>100</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Albuquerque NM</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
         <is>
           <t>2026-10-21</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-21 20:20 UTC (cycle 15)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-21.xlsx
+++ b/output/leads_2026-10-21.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1044,7 +1044,6 @@
           <t>https://albuquerqueroofingpro.com/services/metal-roofing/</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
           <t>ahroofingco28@gmail.com</t>
@@ -1074,6 +1073,122 @@
         </is>
       </c>
       <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Leo Roofing &amp; Construction</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>leoroofingfl.com</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://www.leoroofingfl.com/service-area/port-st-lucie-roofing/</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Palm Beach</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>info@leoroofingfl.com</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>561-935-4979</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Port St Lucie FL</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>100</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>roof replacement Port St Lucie FL</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>OverAll Roofing</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>overallroof.com</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>https://overallroof.com/roof-replacement/</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Free Inspection</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>info@overallroofing.com</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Franklin TN</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>66</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>roof replacement Franklin TN</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
         <is>
           <t>2026-10-21</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-21 20:22 UTC (cycle 16)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-21.xlsx
+++ b/output/leads_2026-10-21.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1169,7 +1169,6 @@
           <t>info@overallroofing.com</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
           <t>Franklin TN</t>
@@ -1189,6 +1188,62 @@
         </is>
       </c>
       <c r="L13" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Anchor Plumbing And Boiler Services</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>anchorplumbingboilerservicesllc.com</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>https://anchorplumbingboilerservicesllc.com/rio-rancho-nm/</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>seanm@anchorplumbingboilerservices.com</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>(505) 803-1134</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Rio Rancho NM</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>76</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>plumber Rio Rancho NM</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
         <is>
           <t>2026-10-21</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-21 20:23 UTC (cycle 17)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-21.xlsx
+++ b/output/leads_2026-10-21.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1214,7 +1214,6 @@
           <t>https://anchorplumbingboilerservicesllc.com/rio-rancho-nm/</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>seanm@anchorplumbingboilerservices.com</t>
@@ -1244,6 +1243,66 @@
         </is>
       </c>
       <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Plumber Austin TX | Leak Detection &amp; Plumbing Experts</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>plumbinatoraustin.com</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>https://www.plumbinatoraustin.com/austin</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Round Rock</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>mickeytheplumber@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>(512) 786-1771</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Austin TX</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>100</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>plumber Austin TX</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
         <is>
           <t>2026-10-21</t>
         </is>

</xml_diff>